<commit_message>
Add 120+ direct career links (Tier 1/2/3) as second sheet in personal Excel
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/personal/PersonalJobs_22062026.xlsx
+++ b/data/personal/PersonalJobs_22062026.xlsx
@@ -508,16 +508,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
     <col width="64" customWidth="1" min="4" max="4"/>
     <col width="31" customWidth="1" min="5" max="5"/>
-    <col width="36" customWidth="1" min="6" max="6"/>
-    <col width="72" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="81" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1">
@@ -530,7 +530,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Report: June 22, 2026 - 03:06 PM | Total: 14</t>
+          <t>Report: June 22, 2026 - 03:31 PM | Total: 26</t>
         </is>
       </c>
     </row>
@@ -583,27 +583,27 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Postman</t>
+          <t>PhonePe</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Data Engineer</t>
+          <t>Site Reliability Engineer 2 - BigData</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bangalore</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>3-5 years, 5 years</t>
+          <t>Fresher</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/postman/jobs/7777990003</t>
+          <t>https://job-boards.greenhouse.io/phonepe/jobs/7771368003</t>
         </is>
       </c>
     </row>
@@ -618,27 +618,27 @@
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>Postman</t>
+          <t>PhonePe</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>Software Engineer, Authorization</t>
+          <t>Site Reliability Engineer 3</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Bangalore</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>3 years, 3 years</t>
+          <t>Fresher</t>
         </is>
       </c>
       <c r="G6" s="10" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/postman/jobs/7776298003</t>
+          <t>https://job-boards.greenhouse.io/phonepe/jobs/7752457003</t>
         </is>
       </c>
     </row>
@@ -648,32 +648,32 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Twilio</t>
+          <t>Postman</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>Software Engineer (L2)</t>
+          <t>Data Engineer</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Remote - India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>3 years</t>
+          <t>Fresher</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/twilio/jobs/7926889</t>
+          <t>https://job-boards.greenhouse.io/postman/jobs/7777990003</t>
         </is>
       </c>
     </row>
@@ -683,32 +683,32 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>New Relic</t>
+          <t>Postman</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>Software Engineer - Fullstack</t>
+          <t>Software Engineer, Authorization</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>Hyderabad, India</t>
+          <t>Bengaluru, Karnataka, India</t>
         </is>
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>2 years, 3 years</t>
+          <t>Fresher</t>
         </is>
       </c>
       <c r="G8" s="10" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/newrelic/jobs/5224725008</t>
+          <t>https://job-boards.greenhouse.io/postman/jobs/7776298003</t>
         </is>
       </c>
     </row>
@@ -718,32 +718,32 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>SingleStore</t>
+          <t>Stripe</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>Software Engineer | AI Platforms</t>
+          <t>Software Engineer, Data &amp; AI</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bengaluru</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>4 years</t>
+          <t>Fresher</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/singlestore/jobs/7573638</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7529428</t>
         </is>
       </c>
     </row>
@@ -753,32 +753,32 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>SingleStore</t>
+          <t>Stripe</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>Software Engineer | Database Engine</t>
+          <t>Software Engineer, Internal Systems</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bengaluru, India</t>
         </is>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t>Not specified (fresher-friendly)</t>
+          <t>Fresher</t>
         </is>
       </c>
       <c r="G10" s="10" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/singlestore/jobs/8000966</t>
+          <t>https://stripe.com/jobs/search?gh_jid=7543868</t>
         </is>
       </c>
     </row>
@@ -788,32 +788,32 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Postman</t>
+          <t>Okta</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>Software Engineer, IAM</t>
+          <t>Software Engineer-Full Stack</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana, India</t>
+          <t>Bengaluru, India</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>3 years, 3 years</t>
+          <t>Fresher</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/postman/jobs/7687341003</t>
+          <t>https://www.okta.com/company/careers/opportunity/7984479?gh_jid=7984479</t>
         </is>
       </c>
     </row>
@@ -823,32 +823,32 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>Notion</t>
+          <t>Rubrik</t>
         </is>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>Software Engineer, Infrastructure</t>
+          <t>Production Engineer/Site Reliability Engineer (Shift Basis)</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>Hyderabad, India</t>
+          <t>Bangalore</t>
         </is>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>4 years, 4 years</t>
+          <t>Fresher</t>
         </is>
       </c>
       <c r="G12" s="10" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/notion/42f18ccd-c4c8-4a85-8c1f-de12c575fe87</t>
+          <t>https://www.rubrik.com/company/careers/departments/job.7439521?gh_jid=7439521</t>
         </is>
       </c>
     </row>
@@ -858,32 +858,32 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Postman</t>
+          <t>New Relic</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>Software Engineer (Fullstack, frontend-heavy), Product Trust</t>
+          <t>Software Engineer - Fullstack</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>Bengaluru, Karnataka, India</t>
+          <t>Hyderabad, India</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>3-5 years, 5 years</t>
+          <t>Fresher</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/postman/jobs/7704063003</t>
+          <t>https://job-boards.greenhouse.io/newrelic/jobs/5224725008</t>
         </is>
       </c>
     </row>
@@ -893,32 +893,32 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>SingleStore</t>
+          <t>Okta</t>
         </is>
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>Software Engineer</t>
+          <t>SRE Operations Engineer</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bengaluru, India</t>
         </is>
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t>4 years</t>
+          <t>Fresher</t>
         </is>
       </c>
       <c r="G14" s="10" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/singlestore/jobs/7967752</t>
+          <t>https://www.okta.com/company/careers/opportunity/8003315?gh_jid=8003315</t>
         </is>
       </c>
     </row>
@@ -928,32 +928,32 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>SingleStore</t>
+          <t>Okta</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>Software Engineer | Cloud Foundations</t>
+          <t>Systems Engineer - Productivity Engineering</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>India (Remote)</t>
+          <t>Bengaluru, India</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>Not specified (fresher-friendly)</t>
+          <t>Fresher</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/singlestore/jobs/7790325</t>
+          <t>https://www.okta.com/company/careers/opportunity/6866775?gh_jid=6866775</t>
         </is>
       </c>
     </row>
@@ -963,32 +963,32 @@
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>SingleStore</t>
+          <t>Adyen</t>
         </is>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>Software Engineer | Engine (Ingest)</t>
+          <t>Machine Learning Engineer</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bengaluru</t>
         </is>
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
-          <t>3-5 years, 3 years</t>
+          <t>Fresher</t>
         </is>
       </c>
       <c r="G16" s="10" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/singlestore/jobs/7868076</t>
+          <t>https://job-boards.greenhouse.io/adyen/jobs/7349167</t>
         </is>
       </c>
     </row>
@@ -998,32 +998,32 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Notion</t>
+          <t>PhonePe</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>Software Engineer, Developer Experience</t>
+          <t>Service Delivery Engineer, SRE</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>Hyderabad, India</t>
+          <t>Bangalore</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>Not specified (fresher-friendly)</t>
+          <t>Fresher</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>https://jobs.ashbyhq.com/notion/49bdf081-6e20-4323-8c73-6d6b19544ff5</t>
+          <t>https://job-boards.greenhouse.io/phonepe/jobs/7762335003</t>
         </is>
       </c>
     </row>
@@ -1033,32 +1033,452 @@
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>ClickHouse</t>
+          <t>PhonePe</t>
         </is>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>Core Software Engineer (C++) - Remote</t>
+          <t>Site Reliability Engineer</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>India (remote)</t>
+          <t>Bangalore</t>
         </is>
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
-          <t>Not specified (fresher-friendly)</t>
+          <t>Fresher</t>
         </is>
       </c>
       <c r="G18" s="10" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/clickhouse/jobs/5767816004</t>
+          <t>https://job-boards.greenhouse.io/phonepe/jobs/7766868003</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>PhonePe</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>Site Reliability Engineer 2</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>Fresher</t>
+        </is>
+      </c>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/phonepe/jobs/7731736003</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="8" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>PhonePe</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>Site Reliability Engineer - Azure (4-8yrs)</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t>Fresher</t>
+        </is>
+      </c>
+      <c r="G20" s="10" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/phonepe/jobs/6589348003</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>Vonage</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>Full Stack Developer III (Vue.js / React.js and Nest.Js)</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>Bangalore, India</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>Fresher</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/vonage/jobs/8518615002</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="8" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>Postman</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>Software Engineer, IAM</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>Hyderabad, Telangana, India</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>Fresher</t>
+        </is>
+      </c>
+      <c r="G22" s="10" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/postman/jobs/7687341003</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>Notion</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>Software Engineer, Infrastructure</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>Hyderabad, India</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>Fresher</t>
+        </is>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/notion/42f18ccd-c4c8-4a85-8c1f-de12c575fe87</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>Vonage</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>Full Stack Software Engineer (C#, JavaScript)</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>Bangalore India</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
+        <is>
+          <t>Fresher</t>
+        </is>
+      </c>
+      <c r="G24" s="10" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/vonage/jobs/8371897002</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>Postman</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>Software Engineer (Fullstack, frontend-heavy), Product Trust</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka, India</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>Fresher</t>
+        </is>
+      </c>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/postman/jobs/7704063003</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="8" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>Anyscale</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>Software Engineer, Platform Infrastructure (Foundations)</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka</t>
+        </is>
+      </c>
+      <c r="F26" s="9" t="inlineStr">
+        <is>
+          <t>Fresher</t>
+        </is>
+      </c>
+      <c r="G26" s="10" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/anyscale/316cf655-f3f1-40c2-823f-34f1fce54fdc</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>Anyscale</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>Software Engineer, Ray Serve</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>Fresher</t>
+        </is>
+      </c>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/anyscale/c35b6d34-710d-4943-85b6-2073ff4eecd1</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="8" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>Notion</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>Software Engineer, Developer Experience</t>
+        </is>
+      </c>
+      <c r="E28" s="9" t="inlineStr">
+        <is>
+          <t>Hyderabad, India</t>
+        </is>
+      </c>
+      <c r="F28" s="9" t="inlineStr">
+        <is>
+          <t>Fresher</t>
+        </is>
+      </c>
+      <c r="G28" s="10" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/notion/49bdf081-6e20-4323-8c73-6d6b19544ff5</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>2025-10-06</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>Anyscale</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>Software Engineer, Ray Core</t>
+        </is>
+      </c>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>Fresher</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/anyscale/8b29c5e5-d56f-4c52-8887-a6a1827cf042</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="8" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>2025-09-10</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>Anyscale</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>Software Engineer, Ray Data</t>
+        </is>
+      </c>
+      <c r="E30" s="9" t="inlineStr">
+        <is>
+          <t>Bengaluru, Karnataka</t>
+        </is>
+      </c>
+      <c r="F30" s="9" t="inlineStr">
+        <is>
+          <t>Fresher</t>
+        </is>
+      </c>
+      <c r="G30" s="10" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/anyscale/2d76cfa2-f857-42b2-9c74-c07beca01458</t>
         </is>
       </c>
     </row>
@@ -1078,6 +1498,18 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId26"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>